<commit_message>
Ne tą PSP įkėliau, įkeliu iš naujo
</commit_message>
<xml_diff>
--- a/PSP.xlsx
+++ b/PSP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Laura/Desktop/2 semestras/Algoritmai ir duomenų struktūros/lab1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Laura/Desktop/2 semestras/Algoritmai ir duomenų struktūros/lab2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E30A0A-7E53-3A41-84C7-72FC7DB6A8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF74B29-7F1B-714C-B8D3-FA384A436FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{5942AB64-4C26-9646-BCDE-E7F2EA838442}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17280" xr2:uid="{5942AB64-4C26-9646-BCDE-E7F2EA838442}"/>
   </bookViews>
   <sheets>
     <sheet name="LFF" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Laura Lukianaitė</t>
   </si>
@@ -71,105 +71,18 @@
     <t>Vnt.</t>
   </si>
   <si>
-    <t>02-21</t>
-  </si>
-  <si>
-    <t>02-22</t>
-  </si>
-  <si>
-    <t>32min</t>
-  </si>
-  <si>
     <t>Skaitymas</t>
   </si>
   <si>
-    <t>Gilinuosi į užduoties reikalavimus, renku informaciją apie deką, sąrašų tipus.</t>
-  </si>
-  <si>
-    <t>Deko eskizas (kokių reikės funkcijų, ką jos darys), paruošiau aplinką, failus.</t>
-  </si>
-  <si>
-    <t>Programavimas + Planavimas</t>
-  </si>
-  <si>
-    <t>13min</t>
-  </si>
-  <si>
     <t>PSP veikla</t>
   </si>
   <si>
-    <t>29min</t>
-  </si>
-  <si>
-    <t>18min</t>
-  </si>
-  <si>
-    <t>19min</t>
-  </si>
-  <si>
     <t>7min</t>
   </si>
   <si>
-    <t>44min</t>
-  </si>
-  <si>
-    <t>Planavimas</t>
-  </si>
-  <si>
     <t>Programavimas</t>
   </si>
   <si>
-    <t>Testavimas</t>
-  </si>
-  <si>
-    <t>Gilinu žinias apie struktūras, rodykles bei mazgus.</t>
-  </si>
-  <si>
-    <t>Funkcijos realizuotos Deque.c faile, main.c failas papildytas visų esamų funkcijų testavimu</t>
-  </si>
-  <si>
-    <t>Su pagalba main.c faile sukurtu testavimo kodu aptikau ir ištaisiau funkcijoje esamas sintaksines bei logines klaidas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sukūriau atskirą failą testavimams test.c, o main.c esantį kodą skyriau demonstraciniams tikslams. Sukurtas Makefile, README.md </t>
-  </si>
-  <si>
-    <t>-10 +170</t>
-  </si>
-  <si>
-    <t>+126</t>
-  </si>
-  <si>
-    <t>+85</t>
-  </si>
-  <si>
-    <t>+20</t>
-  </si>
-  <si>
-    <t>Rašau komentaru, pridedu precondition ir postcondition ten, kur reikia</t>
-  </si>
-  <si>
-    <t>Sukuriu Go.cmd, peržiūriu ar viskas tvarkoje</t>
-  </si>
-  <si>
-    <t>Programavimas + Peržiūra</t>
-  </si>
-  <si>
-    <t>2min</t>
-  </si>
-  <si>
-    <t>12min</t>
-  </si>
-  <si>
-    <t>26min</t>
-  </si>
-  <si>
-    <t>03-02</t>
-  </si>
-  <si>
-    <t>02-23</t>
-  </si>
-  <si>
     <t>Data:</t>
   </si>
   <si>
@@ -179,32 +92,31 @@
     <t>Studentė:</t>
   </si>
   <si>
-    <t>Ant popieriaus lapo paišau deką ir kaip sprendžiu kaip geriausiai realizuoti funkcijas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:22-15:23 Užsinorėjau gerti (sulčių)
-15:35-15:39 Užsimąsčiau apie kažką </t>
-  </si>
-  <si>
-    <t>2h13min</t>
-  </si>
-  <si>
-    <t>16:15-16:20 skambutis</t>
-  </si>
-  <si>
-    <t>40min</t>
-  </si>
-  <si>
-    <t>35min</t>
-  </si>
-  <si>
-    <t>Testavimas + peržiūra</t>
-  </si>
-  <si>
-    <t>Testuoju windows aplinkoje ar viskas pasileidžia, ištaisau klaidas</t>
-  </si>
-  <si>
-    <t>5min</t>
+    <t>03-21</t>
+  </si>
+  <si>
+    <t>Žiūrint į pateiktų pavyzdžių rezultatus, bandau išsiaiškinti dėsningumus karalienių koordinačių kintant trikampės matricos eilučių skaičiui, rašau pseudokodą, braižau ant lapo įvairius atvejus ir tikrinu ar grąžins reikiamą rezultatą mano sprendimo būdas.</t>
+  </si>
+  <si>
+    <t>Projektavimas</t>
+  </si>
+  <si>
+    <t>Skaitau užduotį, gilinu žinias apie backtracking, žiuriu dėstytojų video iš youtube.</t>
+  </si>
+  <si>
+    <t>1h1min</t>
+  </si>
+  <si>
+    <t>47min</t>
+  </si>
+  <si>
+    <t>39min</t>
+  </si>
+  <si>
+    <t>Sukuriu pagrindinius failus. Aprašau .h failą. Remiantis savo pseudokodu, parašau logikos programos dalį n-queen.c faile.</t>
+  </si>
+  <si>
+    <t>+56</t>
   </si>
 </sst>
 </file>
@@ -274,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -297,25 +209,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,393 +565,267 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="11">
+      <c r="A3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="12">
         <v>1</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="H3" s="13" t="s">
-        <v>44</v>
+      <c r="C3" s="12"/>
+      <c r="H3" s="10" t="s">
+        <v>15</v>
       </c>
       <c r="I3" s="2">
-        <v>46074</v>
+        <v>46102</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="11" t="s">
+      <c r="A4" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="11"/>
+      <c r="C4" s="12"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B7" s="5">
-        <v>0.64444444444444449</v>
+        <v>0.51597222222222228</v>
       </c>
       <c r="C7" s="5">
-        <v>0.67361111111111116</v>
+        <v>0.54861111111111116</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="6"/>
     </row>
-    <row r="8" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B8" s="5">
-        <v>0.67361111111111116</v>
+        <v>0.54861111111111116</v>
       </c>
       <c r="C8" s="5">
-        <v>0.70486111111111116</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>50</v>
-      </c>
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H8" s="3"/>
-      <c r="I8" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="I8" s="9"/>
+    </row>
+    <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B9" s="5">
-        <v>0.70486111111111116</v>
+        <v>0.59097222222222223</v>
       </c>
       <c r="C9" s="5">
-        <v>0.71388888888888891</v>
+        <v>0.61805555555555558</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="H9" s="3"/>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="I9" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="4"/>
       <c r="B10" s="5">
-        <v>0.57638888888888884</v>
+        <v>0.61805555555555558</v>
       </c>
       <c r="C10" s="5">
-        <v>0.59652777777777777</v>
+        <v>0.62291666666666667</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>28</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="3"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="5">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0.60972222222222228</v>
-      </c>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
       <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>47</v>
-      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8"/>
       <c r="H11" s="3"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="5">
-        <v>0.60972222222222228</v>
-      </c>
-      <c r="C12" s="5">
-        <v>0.7055555555555556</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>29</v>
-      </c>
+    <row r="12" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5">
-        <v>0.7055555555555556</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0.71875</v>
-      </c>
+      <c r="I12" s="9"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
       <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
       <c r="H13" s="3"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="5">
-        <v>0.71875</v>
-      </c>
-      <c r="C14" s="5">
-        <v>0.72361111111111109</v>
-      </c>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
       <c r="D14" s="6"/>
-      <c r="E14" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>19</v>
-      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="7"/>
       <c r="G14" s="8"/>
       <c r="H14" s="3"/>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="5">
-        <v>0.39305555555555555</v>
-      </c>
-      <c r="C15" s="5">
-        <v>0.4236111111111111</v>
-      </c>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="5">
-        <v>0.4236111111111111</v>
-      </c>
-      <c r="C16" s="5">
-        <v>0.42499999999999999</v>
-      </c>
+      <c r="I15" s="9"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="4"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
       <c r="D16" s="6"/>
-      <c r="E16" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>19</v>
-      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="7"/>
       <c r="G16" s="8"/>
       <c r="H16" s="3"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="5">
-        <v>0.88194444444444442</v>
-      </c>
-      <c r="C17" s="5">
-        <v>0.89027777777777772</v>
-      </c>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
       <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="E17" s="6"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
       <c r="H17" s="3"/>
-      <c r="I17" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="5">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="C18" s="5">
-        <v>0.53888888888888886</v>
-      </c>
+      <c r="I17" s="9"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="4"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
       <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
       <c r="H18" s="3"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="5">
-        <v>0.89583333333333337</v>
-      </c>
-      <c r="C19" s="5">
-        <v>0.92013888888888884</v>
-      </c>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="4"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
       <c r="D19" s="3"/>
-      <c r="E19" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>54</v>
-      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="8"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="5">
-        <v>0.92013888888888884</v>
-      </c>
-      <c r="C20" s="5">
-        <v>0.92361111111111116</v>
-      </c>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
       <c r="D20" s="3"/>
-      <c r="E20" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>19</v>
-      </c>
+      <c r="E20" s="6"/>
+      <c r="F20" s="7"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>

</xml_diff>

<commit_message>
Iki galo dabaigta ir atsiskaityti užduotis
</commit_message>
<xml_diff>
--- a/PSP.xlsx
+++ b/PSP.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Laura/Desktop/2 semestras/Algoritmai ir duomenų struktūros/lab2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF74B29-7F1B-714C-B8D3-FA384A436FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB9CF39-678D-7443-9451-66FE84B119E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17280" xr2:uid="{5942AB64-4C26-9646-BCDE-E7F2EA838442}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="15140" windowHeight="17800" xr2:uid="{5942AB64-4C26-9646-BCDE-E7F2EA838442}"/>
   </bookViews>
   <sheets>
     <sheet name="LFF" sheetId="1" r:id="rId1"/>
+    <sheet name="DFF" sheetId="2" r:id="rId2"/>
+    <sheet name="DTS" sheetId="3" r:id="rId3"/>
+    <sheet name="KPS" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="121">
   <si>
     <t>Laura Lukianaitė</t>
   </si>
@@ -117,13 +120,310 @@
   </si>
   <si>
     <t>+56</t>
+  </si>
+  <si>
+    <t>03-22</t>
+  </si>
+  <si>
+    <t>23 min</t>
+  </si>
+  <si>
+    <t>Pabaigta rašyti logikos programos dalis, main.c</t>
+  </si>
+  <si>
+    <t>+29</t>
+  </si>
+  <si>
+    <t>Testavimas</t>
+  </si>
+  <si>
+    <t>28min</t>
+  </si>
+  <si>
+    <t>Tikrinu ar teisingai gavosi rezultatas</t>
+  </si>
+  <si>
+    <t>03-23</t>
+  </si>
+  <si>
+    <t>12min</t>
+  </si>
+  <si>
+    <t>Porgramavimas</t>
+  </si>
+  <si>
+    <t>Taisau kodą, formatuoju tinkamą išvedimą.</t>
+  </si>
+  <si>
+    <t>+18</t>
+  </si>
+  <si>
+    <t>10 min pertrauka</t>
+  </si>
+  <si>
+    <t>54min</t>
+  </si>
+  <si>
+    <t>Pridedu -timeout jei skaičiai darosi didesni</t>
+  </si>
+  <si>
+    <t>+45</t>
+  </si>
+  <si>
+    <t>main.c faila pakeičiu, jog atitiktų užduoties reikalavimus.</t>
+  </si>
+  <si>
+    <t>README.md, Makefile, Go.cmd kūrimas</t>
+  </si>
+  <si>
+    <t>56min</t>
+  </si>
+  <si>
+    <t>30min</t>
+  </si>
+  <si>
+    <t>Radimo data</t>
+  </si>
+  <si>
+    <t>Defekto numeris</t>
+  </si>
+  <si>
+    <t>Defekto tipas</t>
+  </si>
+  <si>
+    <t>Padarytas fazėje</t>
+  </si>
+  <si>
+    <t>Pašalintas fazėje</t>
+  </si>
+  <si>
+    <t>Taisymo laikas</t>
+  </si>
+  <si>
+    <t>Taisant defektą</t>
+  </si>
+  <si>
+    <t>Detalus defekto aprašas</t>
+  </si>
+  <si>
+    <t>Defektų tipų Standartas</t>
+  </si>
+  <si>
+    <t>Tipo numeris</t>
+  </si>
+  <si>
+    <t>Tipo pavadinimas</t>
+  </si>
+  <si>
+    <t>Aprašas</t>
+  </si>
+  <si>
+    <t>Dokumentavimas</t>
+  </si>
+  <si>
+    <t>komentarai, pranešimai</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>comments, messages</t>
+  </si>
+  <si>
+    <t>Sintaksė</t>
+  </si>
+  <si>
+    <t>sintaksinės klaidos</t>
+  </si>
+  <si>
+    <t>Syntax</t>
+  </si>
+  <si>
+    <t>spelling, punctuation, typos, instruction formats</t>
+  </si>
+  <si>
+    <t>Versijavimas</t>
+  </si>
+  <si>
+    <t>pakeitimų valdymas, versijų kontrolė</t>
+  </si>
+  <si>
+    <t>Build, package</t>
+  </si>
+  <si>
+    <t>change management, library, version control</t>
+  </si>
+  <si>
+    <t>Vardai</t>
+  </si>
+  <si>
+    <t>aprašai, vienodi vardai, galiojimo sritis</t>
+  </si>
+  <si>
+    <t>Assignment</t>
+  </si>
+  <si>
+    <t>declaration, duplicate names, scope, limits</t>
+  </si>
+  <si>
+    <t>Interfeisas</t>
+  </si>
+  <si>
+    <t>funkcijų/procedūrų iškvietimai, įvedimas-išvedimas, vartotojo formatai</t>
+  </si>
+  <si>
+    <t>Interface</t>
+  </si>
+  <si>
+    <t>procedure calls and references, I/O, user formats</t>
+  </si>
+  <si>
+    <t>Kontrolė</t>
+  </si>
+  <si>
+    <t>klaidų pranešimai, nepakankama kontrolė</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>error messages, inadequate checks</t>
+  </si>
+  <si>
+    <t>Duomenys</t>
+  </si>
+  <si>
+    <t>duomenų struktūros ir turinys</t>
+  </si>
+  <si>
+    <t>structure, contents</t>
+  </si>
+  <si>
+    <t>Funkcionalumas</t>
+  </si>
+  <si>
+    <t>logika, rodyklės, ciklai, rekursija, skaičiavimai, funkcionalumo defektai</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>logic, pointers, loops, recursion, computation, function defects</t>
+  </si>
+  <si>
+    <t>Sistema</t>
+  </si>
+  <si>
+    <t>konfigūracija, sinchronizavimas, atminties valdymas</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>configuration, timing, memory</t>
+  </si>
+  <si>
+    <t>Aplinka</t>
+  </si>
+  <si>
+    <t>aplinkos (projektavimo, kompiliavimo, testavimo ar kt.) problemos</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>design, compile, test, or other support system problems</t>
+  </si>
+  <si>
+    <t>Kodo peržiūros standartas</t>
+  </si>
+  <si>
+    <t>Aspektas</t>
+  </si>
+  <si>
+    <t>Tikrinami punktai</t>
+  </si>
+  <si>
+    <t>Rasta defektų</t>
+  </si>
+  <si>
+    <t>Išbaigtumas</t>
+  </si>
+  <si>
+    <t>Inicializacija</t>
+  </si>
+  <si>
+    <t>Funkcijų iškvietimas</t>
+  </si>
+  <si>
+    <t>{} poros</t>
+  </si>
+  <si>
+    <t>Patikrinti blokų struktūrą:
+- Ar visi ciklai ir if sąlygos turi teisingai uždarytus skliaustelius.
+- Ar kodo lygiavimas (indentation) atitinka blokus.</t>
+  </si>
+  <si>
+    <t>Loginiai operatoriai</t>
+  </si>
+  <si>
+    <t>Atminties valdymas</t>
+  </si>
+  <si>
+    <t>Standartai</t>
+  </si>
+  <si>
+    <t>Patikrinti, ar programos kodas atitinka naudojamą Kodavimo standartą</t>
+  </si>
+  <si>
+    <t>Failai</t>
+  </si>
+  <si>
+    <t>Patikrinti I/O operacijas:
+- Ar failas atidaromas (fopen).
+- Ar tikrinama, ar failas egzistuoja.
+- Ar failas uždaromas (fclose).</t>
+  </si>
+  <si>
+    <t>Viso</t>
+  </si>
+  <si>
+    <t>Patikrinti, ar realizuotos visos užduoties dalys:
+- M-valdovių dėstymas N trikampėje matricoje
+- Duomenų nuskaitymas iš failo</t>
+  </si>
+  <si>
+    <t>Patikrinti, ar:
+- Masyvai yra tinkamai nunulinti.
+- Kintamieji (totalNodes, limitReached) inicializuoti prieš naudojimą.</t>
+  </si>
+  <si>
+    <t>Patikrinti rodyklių ir adresų perdavimą:
+- Ar perduodant adresą į scanf naudojama reikiama dereferencija (* arba &amp;).
+- Ar funkcijos, turinčios grąžinti duomenis, tai daro korektiškai.</t>
+  </si>
+  <si>
+    <t>Patikrinti kintamųjų ir funkcijų pavadinimus:
+- Ar pavadinimai informatyvūs (queensPlaced, rStart, limitReached).
+- Ar laikomasi vieningo stiliaus (camelCase arba snake_case).</t>
+  </si>
+  <si>
+    <t>Patikrinti algoritmą:
+- Ar vidiniai ciklai neperžengia masyvo ribų (OOB - Out of Bounds).
+- Ar teisingai naudojamos palyginimo sąlygos.</t>
+  </si>
+  <si>
+    <t>malloc nenaudojama</t>
+  </si>
+  <si>
+    <t>9min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -150,16 +450,54 @@
       <color theme="1"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="27"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -182,11 +520,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -219,6 +594,106 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -702,7 +1177,9 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
+      <c r="A10" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="B10" s="5">
         <v>0.61805555555555558</v>
       </c>
@@ -720,79 +1197,169 @@
       <c r="H10" s="3"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+    <row r="11" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="5">
+        <v>0.70625000000000004</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.68055555555555558</v>
+      </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+      <c r="E11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>29</v>
+      </c>
       <c r="H11" s="3"/>
-      <c r="I11" s="6"/>
+      <c r="I11" s="9" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
+      <c r="A12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="5">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.7</v>
+      </c>
       <c r="D12" s="8"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+      <c r="E12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="H12" s="3"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
+    <row r="13" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="5">
+        <v>0.58125000000000004</v>
+      </c>
+      <c r="C13" s="5">
+        <v>0.58958333333333335</v>
+      </c>
       <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8"/>
+      <c r="E13" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>37</v>
+      </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="6"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="8"/>
+      <c r="I13" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="5">
+        <v>0.6118055555555556</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0.65625</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>41</v>
+      </c>
       <c r="H14" s="3"/>
-      <c r="I14" s="6"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
+      <c r="I14" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="5">
+        <v>0.84375</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0.88263888888888886</v>
+      </c>
       <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="8"/>
+      <c r="E15" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="H15" s="3"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
+    <row r="16" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="5">
+        <v>0.88263888888888886</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0.90347222222222223</v>
+      </c>
       <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="8"/>
+      <c r="E16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>44</v>
+      </c>
       <c r="H16" s="3"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
+    <row r="17" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="5">
+        <v>0.90347222222222223</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0.90972222222222221</v>
+      </c>
       <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="7"/>
+      <c r="E17" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="G17" s="8"/>
       <c r="H17" s="3"/>
       <c r="I17" s="9"/>
@@ -887,4 +1454,786 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939D01F4-4063-B440-9D15-0B93C66EF7EC}">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="42" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="18"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="19"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="17"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="19"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="19"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="19"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="19"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="19"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="19"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="19"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="19"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="19"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="19"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="19"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="19"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="19"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="19"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="19"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="19"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="19"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="19"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="19"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="19"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="19"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="19"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="19"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="17"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="19"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="17"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="19"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="17"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="19"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Klaida" error="Fazę reikia pasirinkti!" promptTitle="Pasirinkite" prompt="fazę" sqref="D2:E31" xr:uid="{398E446E-E159-764C-A56E-0DF076116F5C}">
+      <formula1>$J$6:$J$12</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB6339F-93E1-2F4B-BA7C-4E8329A115BB}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="3" max="3" width="29.5" customWidth="1"/>
+    <col min="4" max="4" width="29.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+    </row>
+    <row r="2" spans="1:7" ht="42" x14ac:dyDescent="0.2">
+      <c r="B2" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="22"/>
+    </row>
+    <row r="3" spans="1:7" ht="26" x14ac:dyDescent="0.2">
+      <c r="B3" s="23">
+        <v>10</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="22"/>
+      <c r="F3" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="26" x14ac:dyDescent="0.2">
+      <c r="B4" s="23">
+        <v>20</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="22"/>
+      <c r="F4" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="52" x14ac:dyDescent="0.2">
+      <c r="B5" s="23">
+        <v>30</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="22"/>
+      <c r="F5" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="52" x14ac:dyDescent="0.2">
+      <c r="B6" s="23">
+        <v>40</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="22"/>
+      <c r="F6" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="91" x14ac:dyDescent="0.2">
+      <c r="B7" s="23">
+        <v>50</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="22"/>
+      <c r="F7" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="52" x14ac:dyDescent="0.2">
+      <c r="B8" s="23">
+        <v>60</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="22"/>
+      <c r="F8" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="39" x14ac:dyDescent="0.2">
+      <c r="B9" s="23">
+        <v>70</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="22"/>
+      <c r="F9" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="91" x14ac:dyDescent="0.2">
+      <c r="B10" s="23">
+        <v>80</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="22"/>
+      <c r="F10" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="65" x14ac:dyDescent="0.2">
+      <c r="B11" s="23">
+        <v>90</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="22"/>
+      <c r="F11" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="78" x14ac:dyDescent="0.2">
+      <c r="B12" s="23">
+        <v>100</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="22"/>
+      <c r="F12" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B86A08-903F-554E-80CB-91DBD6DA0B38}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="38.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="20"/>
+    </row>
+    <row r="2" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="B2" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="28"/>
+      <c r="E2" s="15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="53" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="31"/>
+      <c r="E3" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="33"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="35"/>
+    </row>
+    <row r="5" spans="1:5" ht="77" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="D5" s="37"/>
+      <c r="E5" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6" s="33"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="35"/>
+    </row>
+    <row r="7" spans="1:5" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="37"/>
+      <c r="E7" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="35"/>
+    </row>
+    <row r="9" spans="1:5" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="37"/>
+      <c r="E9" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="35"/>
+    </row>
+    <row r="11" spans="1:5" ht="77" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="31"/>
+      <c r="E11" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12" s="33"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="35"/>
+    </row>
+    <row r="13" spans="1:5" ht="87" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="37"/>
+      <c r="E13" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B14" s="33"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="35"/>
+    </row>
+    <row r="15" spans="1:5" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="37"/>
+      <c r="E15" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" s="33"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="35"/>
+    </row>
+    <row r="17" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="35"/>
+    </row>
+    <row r="19" spans="2:5" ht="69" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" s="37"/>
+      <c r="E19" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B20" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="41"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="43">
+        <f>SUM(E3:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="C7:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>